<commit_message>
feat: room util bar extends to all Y modes containing Room
- _draw_cell_util_bars: guard changed from y_dims==["Room"] to "Room" in y_dims
- _build_layout_and_heights: CELL_UTIL_H reserved for any mode with Room dim
- extract room code from row key using room_dim_idx (handles SKU|Room, SO|Room etc.)
- mouseMoveEvent: util bar tooltip shows planned/capacity inner units + % on hover

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/06_CRP.xlsx
+++ b/06_CRP.xlsx
@@ -1375,10 +1375,10 @@
         <v>100</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="K2" s="2" t="n">
         <v>80</v>
@@ -1420,22 +1420,22 @@
         <v>90</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="Z2" s="2" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AD2" s="2" t="n">
         <v>0</v>

</xml_diff>